<commit_message>
notas projetos... junho corrigidas, ok
</commit_message>
<xml_diff>
--- a/05 Others/2026.1 Avaliação Projetos/Turma Engenharia de Software - ARA0097 Turma 3003  SEMI Wyden UniRuy 2026_1.xlsx
+++ b/05 Others/2026.1 Avaliação Projetos/Turma Engenharia de Software - ARA0097 Turma 3003  SEMI Wyden UniRuy 2026_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\Avaliações Yduqs 2022_2 BDQ 2023_1 2024_2\2026.1 Avaliação Projetos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19165AB-D04C-4335-AB06-9FD1218869B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D7F70A-AE96-4004-B7EE-275A945814B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD6ED3E7-57DF-4A52-9E4C-63B0F7661B3D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>AV</t>
   </si>
@@ -95,7 +95,61 @@
     <t>FIGMA; https://projeto-eng-software.vercel.app/</t>
   </si>
   <si>
-    <t>https://cinebrbrasil.netlify.app/</t>
+    <t>não</t>
+  </si>
+  <si>
+    <t>Peso AV 8</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>não ABNT</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+https://cinebrbrasil.netlify.app/</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>não apresentou o projeto de eng de software, somente o descritivo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+FIGMA; https://projeto-eng-software.vercel.app/</t>
+    </r>
+  </si>
+  <si>
+    <t>Não fez nada do projeto de eng de soft</t>
   </si>
 </sst>
 </file>
@@ -105,7 +159,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +213,36 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -186,7 +270,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -377,45 +461,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -424,7 +469,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -445,15 +490,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -466,20 +505,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -492,7 +519,26 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -837,17 +883,18 @@
     <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="54.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="5" t="s">
@@ -876,46 +923,51 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="9">
+      <c r="B2" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="D2" s="8">
         <v>0</v>
       </c>
-      <c r="D2" s="9">
+      <c r="E2" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="F2" s="8">
+        <v>1</v>
+      </c>
+      <c r="G2" s="20">
+        <f>C2/8*4</f>
+        <v>3.6</v>
+      </c>
+      <c r="H2" s="14">
         <v>0</v>
       </c>
-      <c r="E2" s="9">
-        <v>0.9</v>
-      </c>
-      <c r="F2" s="9">
-        <v>1</v>
-      </c>
-      <c r="G2" s="10">
-        <f>$C$2*7/4</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="20">
-        <v>0</v>
-      </c>
-      <c r="I2" s="11">
+      <c r="I2" s="9">
         <f>G2+H2</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="24" t="s">
+        <v>3.6</v>
+      </c>
+      <c r="J2" s="18" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="K2" s="24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="7">
         <v>7</v>
       </c>
       <c r="C3" s="7">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="D3" s="7">
         <v>0</v>
@@ -926,33 +978,33 @@
       <c r="F3" s="7">
         <v>0.4</v>
       </c>
-      <c r="G3" s="8">
-        <f t="shared" ref="G3:G5" si="0">$C$2*7/4</f>
-        <v>0</v>
+      <c r="G3" s="21">
+        <f t="shared" ref="G3:G5" si="0">C3/8*4</f>
+        <v>3.2</v>
       </c>
       <c r="H3" s="1">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I5" si="1">G3+H3</f>
         <v>6</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="J3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="K3" t="s">
-        <v>18</v>
+      <c r="K3" s="26" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="7">
         <v>7</v>
       </c>
       <c r="C4" s="7">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="D4" s="7">
         <v>0</v>
@@ -963,59 +1015,59 @@
       <c r="F4" s="7">
         <v>0.6</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="21">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H4" s="1">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="15" t="s">
         <v>15</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="12">
         <v>5</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="12">
+        <v>7.2</v>
+      </c>
+      <c r="D5" s="12">
         <v>0</v>
       </c>
-      <c r="D5" s="14">
-        <v>0</v>
-      </c>
-      <c r="E5" s="14">
+      <c r="E5" s="12">
         <v>0.7</v>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="12">
         <v>0.5</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="22">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H5" s="2">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="I5" s="2">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J5" s="22" t="s">
+        <v>9.1</v>
+      </c>
+      <c r="J5" s="16" t="s">
         <v>16</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1029,7 +1081,9 @@
         <v>9</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="C7" s="23" t="s">
+        <v>20</v>
+      </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1103,7 +1157,7 @@
     <hyperlink ref="J3" r:id="rId1" xr:uid="{14378773-7BD9-4DE3-9688-86AA7688AD4F}"/>
     <hyperlink ref="J4" r:id="rId2" xr:uid="{CF8E7ADA-2BA6-4571-AA09-0B913E6A2E6C}"/>
     <hyperlink ref="J5" r:id="rId3" xr:uid="{3DEB873A-8F27-41E4-9A86-6244BFA2F083}"/>
-    <hyperlink ref="K5" r:id="rId4" xr:uid="{63EB79D3-AD0C-4CD4-9A1F-BEF5ACDFF254}"/>
+    <hyperlink ref="K5" r:id="rId4" display="https://cinebrbrasil.netlify.app/" xr:uid="{63EB79D3-AD0C-4CD4-9A1F-BEF5ACDFF254}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>

</xml_diff>